<commit_message>
Automatiza 73 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
@@ -340,7 +340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1863,6 +1863,586 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>0,75 Nest 1</t>
+        </is>
+      </c>
+      <c r="D53" s="2">
+        <f>E53/21</f>
+        <v/>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>001574</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>0,75 Nest 2</t>
+        </is>
+      </c>
+      <c r="D54" s="2">
+        <f>E54/21</f>
+        <v/>
+      </c>
+      <c r="E54" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>001575</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>0,75 Nest 3</t>
+        </is>
+      </c>
+      <c r="D55" s="2">
+        <f>E55/21</f>
+        <v/>
+      </c>
+      <c r="E55" t="n">
+        <v>7</v>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>001576</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>0,75 Nest 4</t>
+        </is>
+      </c>
+      <c r="D56" s="2">
+        <f>E56/21</f>
+        <v/>
+      </c>
+      <c r="E56" t="n">
+        <v>14</v>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>001577</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>0,75 Nest 5</t>
+        </is>
+      </c>
+      <c r="D57" s="2">
+        <f>E57/21</f>
+        <v/>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>001578</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>0,75 Nest 6</t>
+        </is>
+      </c>
+      <c r="D58" s="2">
+        <f>E58/21</f>
+        <v/>
+      </c>
+      <c r="E58" t="n">
+        <v>5</v>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>001579</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>0,75 Nest 7</t>
+        </is>
+      </c>
+      <c r="D59" s="2">
+        <f>E59/21</f>
+        <v/>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>001580</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>0,75 Nest 8</t>
+        </is>
+      </c>
+      <c r="D60" s="2">
+        <f>E60/21</f>
+        <v/>
+      </c>
+      <c r="E60" t="n">
+        <v>4</v>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>001581</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>0,75 Nest 9</t>
+        </is>
+      </c>
+      <c r="D61" s="2">
+        <f>E61/21</f>
+        <v/>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>001582</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>0,9 Nest 1</t>
+        </is>
+      </c>
+      <c r="D62" s="2">
+        <f>E62/21</f>
+        <v/>
+      </c>
+      <c r="E62" t="n">
+        <v>21</v>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>001583</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>0,9 Nest 2</t>
+        </is>
+      </c>
+      <c r="D63" s="2">
+        <f>E63/21</f>
+        <v/>
+      </c>
+      <c r="E63" t="n">
+        <v>14</v>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>001584</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>0,9 Nest 3</t>
+        </is>
+      </c>
+      <c r="D64" s="2">
+        <f>E64/21</f>
+        <v/>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>001585</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>0,9 Nest 4</t>
+        </is>
+      </c>
+      <c r="D65" s="2">
+        <f>E65/21</f>
+        <v/>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>001586</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>0,9 Nest 5</t>
+        </is>
+      </c>
+      <c r="D66" s="2">
+        <f>E66/21</f>
+        <v/>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>001587</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>0,9 Nest 6</t>
+        </is>
+      </c>
+      <c r="D67" s="2">
+        <f>E67/21</f>
+        <v/>
+      </c>
+      <c r="E67" t="n">
+        <v>31</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>001588</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>0,9 Nest 7</t>
+        </is>
+      </c>
+      <c r="D68" s="2">
+        <f>E68/21</f>
+        <v/>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>001589</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2,65 Nest 1</t>
+        </is>
+      </c>
+      <c r="D69" s="2">
+        <f>E69/21</f>
+        <v/>
+      </c>
+      <c r="E69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>001590</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2,65 Nest 2</t>
+        </is>
+      </c>
+      <c r="D70" s="2">
+        <f>E70/21</f>
+        <v/>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>001591</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2,65 Nest 3</t>
+        </is>
+      </c>
+      <c r="D71" s="2">
+        <f>E71/21</f>
+        <v/>
+      </c>
+      <c r="E71" t="n">
+        <v>4</v>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>001592</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Laser Chapa</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2,65 Nest 4</t>
+        </is>
+      </c>
+      <c r="D72" s="2">
+        <f>E72/21</f>
+        <v/>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>001593</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Automatiza 92 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -27,6 +27,10 @@
       <name val="Carlito"/>
       <color rgb="FF17313A"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
@@ -340,13 +344,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="6"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="11"/>
@@ -2443,6 +2447,538 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Chapa Parachoque</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>21</v>
+      </c>
+      <c r="E73" t="n">
+        <v>8</v>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>001594</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Bdj Central Dobra</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>21</v>
+      </c>
+      <c r="E74" t="n">
+        <v>3</v>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>001595</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bdj Lat Maior Dobra</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>21</v>
+      </c>
+      <c r="E75" t="n">
+        <v>8</v>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>001596</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bdj Lat Menor Dobra</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>21</v>
+      </c>
+      <c r="E76" t="n">
+        <v>4</v>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>001597</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bdj Lat Menor Amassamento</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>21</v>
+      </c>
+      <c r="E77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>001598</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Fechamento testeira</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>21</v>
+      </c>
+      <c r="E78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>001599</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Trava S</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>21</v>
+      </c>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>001600</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Fechamento lat menor</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>21</v>
+      </c>
+      <c r="E80" t="n">
+        <v>4</v>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>001601</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Fechamento lat médio</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>21</v>
+      </c>
+      <c r="E81" t="n">
+        <v>6</v>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>001602</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Fechamento lateral</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>21</v>
+      </c>
+      <c r="E82" t="n">
+        <v>4</v>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>001603</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Fechamento lat maior</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>21</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>001604</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Encaixe Central</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>21</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>001605</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Encaixe Lateral</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>21</v>
+      </c>
+      <c r="E85" t="n">
+        <v>4</v>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>001606</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Trava Estrutura Central</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>21</v>
+      </c>
+      <c r="E86" t="n">
+        <v>4</v>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>001607</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Lateral Tampa</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>21</v>
+      </c>
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>001608</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Fundo Maior</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>21</v>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>001609</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>L 350mm</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>21</v>
+      </c>
+      <c r="E89" t="n">
+        <v>4</v>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>001610</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>L 460mm</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>21</v>
+      </c>
+      <c r="E90" t="n">
+        <v>8</v>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>001611</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Dobradeira de Chapas</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>L 970mm</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>21</v>
+      </c>
+      <c r="E91" t="n">
+        <v>4</v>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>001612</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Automatiza 110 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG BACKLIGHT MODELO 1.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2464,10 +2464,10 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
@@ -2492,10 +2492,10 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
@@ -2520,10 +2520,10 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
@@ -2548,10 +2548,10 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
@@ -2576,10 +2576,10 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
@@ -2604,10 +2604,10 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
@@ -2632,10 +2632,10 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
@@ -2660,10 +2660,10 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
@@ -2688,10 +2688,10 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="E81" t="n">
-        <v>6</v>
+        <v>126</v>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
@@ -2716,10 +2716,10 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
@@ -2744,10 +2744,10 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
@@ -2772,10 +2772,10 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
@@ -2828,10 +2828,10 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
@@ -2856,10 +2856,10 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>42</v>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         </is>
       </c>
       <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="n">
         <v>21</v>
-      </c>
-      <c r="E88" t="n">
-        <v>1</v>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
@@ -2912,10 +2912,10 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>84</v>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
@@ -2940,10 +2940,10 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E90" t="n">
-        <v>8</v>
+        <v>168</v>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
@@ -2968,14 +2968,518 @@
         </is>
       </c>
       <c r="D91" t="n">
+        <v>4</v>
+      </c>
+      <c r="E91" t="n">
+        <v>84</v>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>001612</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LE</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
         <v>21</v>
       </c>
-      <c r="E91" t="n">
-        <v>4</v>
-      </c>
-      <c r="F91" s="3" t="inlineStr">
-        <is>
-          <t>001612</t>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>001613</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LD</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" t="n">
+        <v>21</v>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>001614</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Quadro Testeira</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>2</v>
+      </c>
+      <c r="E94" t="n">
+        <v>42</v>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>001615</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Testeira</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" t="n">
+        <v>21</v>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>001616</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Canaleta Testeira</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" t="n">
+        <v>21</v>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>001617</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Corpo Central</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="n">
+        <v>21</v>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>001618</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Trava Corpo Central</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="n">
+        <v>21</v>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>001619</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Esq</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" t="n">
+        <v>21</v>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>001620</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Dir</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="n">
+        <v>21</v>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>001621</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Cruzeta</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>2</v>
+      </c>
+      <c r="E101" t="n">
+        <v>42</v>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>001622</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Parachoque</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>2</v>
+      </c>
+      <c r="E102" t="n">
+        <v>42</v>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>001623</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Chapa do rodizio corpo lateral</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" t="n">
+        <v>42</v>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>001624</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Bdj Maior Lateral</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>8</v>
+      </c>
+      <c r="E104" t="n">
+        <v>168</v>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>001625</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Maior Lat</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>8</v>
+      </c>
+      <c r="E105" t="n">
+        <v>168</v>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>001626</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Bdj Menor Lateral</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>2</v>
+      </c>
+      <c r="E106" t="n">
+        <v>42</v>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>001627</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Menor Lat</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>2</v>
+      </c>
+      <c r="E107" t="n">
+        <v>42</v>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>001628</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Bdj Central</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>2</v>
+      </c>
+      <c r="E108" t="n">
+        <v>42</v>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>001629</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 1</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Central</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>2</v>
+      </c>
+      <c r="E109" t="n">
+        <v>42</v>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>001630</t>
         </is>
       </c>
     </row>

</xml_diff>